<commit_message>
Facitliste, tabeller og layout rettet.
</commit_message>
<xml_diff>
--- a/undervisningsforlob/valg_af_parti/datasæt_4_personer.xlsx
+++ b/undervisningsforlob/valg_af_parti/datasæt_4_personer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aalbcitygym-my.sharepoint.com/personal/js_aacg_dk/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\Documents\GitHub\aalborg-intelligence.github.io\undervisningsforlob\valg_af_parti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18A66C14-3C4B-4837-8AB8-D8CB986CD545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8B1D68-A1E3-4314-8584-5D811444E182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0E262B79-17A8-45B4-B858-31DA2D8D6D5E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{0E262B79-17A8-45B4-B858-31DA2D8D6D5E}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Person</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>t</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -95,8 +104,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,9 +442,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51CA511-2210-430E-B64D-3E12A1C59EFE}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -448,60 +458,60 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>-2</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>-2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C3" s="1">
         <v>1</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>-1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>-1</v>
-      </c>
-      <c r="C4">
-        <v>-1</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>